<commit_message>
Mixed simulation with shifts.
</commit_message>
<xml_diff>
--- a/backend/ProductionPlanning_v6.xlsx
+++ b/backend/ProductionPlanning_v6.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\paa7bue\Documents\UseCases\backend\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Alex\Master\2026 SS\Masterarbeit\phase 3\backend\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1B876ED2-F951-44FC-A175-4AB690D4FA5C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CFCF7C52-AAC4-4743-8EE5-A43316227421}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" tabRatio="580" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" tabRatio="580" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Process" sheetId="1" r:id="rId1"/>
@@ -29,28 +29,15 @@
     <sheet name="README" sheetId="8" r:id="rId14"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">CustomerDemand!$A$3:$E$22</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">CustomerDemandKanban!$A$2:$B$23</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">CustomerDemand!$A$3:$E$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">CustomerDemandKanban!$A$2:$B$8</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
-  <extLst>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
-  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="867" uniqueCount="280">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1056" uniqueCount="323">
   <si>
     <t>PROCESS PARAMETERS</t>
   </si>
@@ -800,9 +787,6 @@
     <t>14:52:13</t>
   </si>
   <si>
-    <t>09:39:02</t>
-  </si>
-  <si>
     <t>14:13:29</t>
   </si>
   <si>
@@ -884,13 +868,145 @@
     <t>Ends</t>
   </si>
   <si>
-    <t>extra</t>
-  </si>
-  <si>
-    <t>ex</t>
-  </si>
-  <si>
-    <t>camb</t>
+    <t>07:20:11</t>
+  </si>
+  <si>
+    <t>16:55:20</t>
+  </si>
+  <si>
+    <t>19:18:13</t>
+  </si>
+  <si>
+    <t>04:20:09</t>
+  </si>
+  <si>
+    <t>10:41:32</t>
+  </si>
+  <si>
+    <t>16:01:58</t>
+  </si>
+  <si>
+    <t>09.09.2026</t>
+  </si>
+  <si>
+    <t>08:00:56</t>
+  </si>
+  <si>
+    <t>10:03:53</t>
+  </si>
+  <si>
+    <t>12:41:56</t>
+  </si>
+  <si>
+    <t>16:37:56</t>
+  </si>
+  <si>
+    <t>10.09.2026</t>
+  </si>
+  <si>
+    <t>03:47:01</t>
+  </si>
+  <si>
+    <t>05:09:54</t>
+  </si>
+  <si>
+    <t>13:13:36</t>
+  </si>
+  <si>
+    <t>11.09.2026</t>
+  </si>
+  <si>
+    <t>05:18:46</t>
+  </si>
+  <si>
+    <t>12.09.2026</t>
+  </si>
+  <si>
+    <t>00:26:24</t>
+  </si>
+  <si>
+    <t>04:42:03</t>
+  </si>
+  <si>
+    <t>04:56:04</t>
+  </si>
+  <si>
+    <t>14.09.2026</t>
+  </si>
+  <si>
+    <t>14:42:13</t>
+  </si>
+  <si>
+    <t>17:52:37</t>
+  </si>
+  <si>
+    <t>20:47:25</t>
+  </si>
+  <si>
+    <t>21:41:01</t>
+  </si>
+  <si>
+    <t>15.09.2026</t>
+  </si>
+  <si>
+    <t>08:11:47</t>
+  </si>
+  <si>
+    <t>09:25:30</t>
+  </si>
+  <si>
+    <t>13:38:22</t>
+  </si>
+  <si>
+    <t>14:21:48</t>
+  </si>
+  <si>
+    <t>18:51:29</t>
+  </si>
+  <si>
+    <t>11:13:45</t>
+  </si>
+  <si>
+    <t>21:17:59</t>
+  </si>
+  <si>
+    <t>05:39:20</t>
+  </si>
+  <si>
+    <t>13:13:24</t>
+  </si>
+  <si>
+    <t>10:22:21</t>
+  </si>
+  <si>
+    <t>16:46:48</t>
+  </si>
+  <si>
+    <t>17:11:02</t>
+  </si>
+  <si>
+    <t>01:24:23</t>
+  </si>
+  <si>
+    <t>04:59:43</t>
+  </si>
+  <si>
+    <t>14:13:44</t>
+  </si>
+  <si>
+    <t>16:04:32</t>
+  </si>
+  <si>
+    <t>14:56:47</t>
+  </si>
+  <si>
+    <t>05:12:28</t>
+  </si>
+  <si>
+    <t>15:19:03</t>
+  </si>
+  <si>
+    <t>22:04:50</t>
   </si>
 </sst>
 </file>
@@ -1143,7 +1259,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="59">
+  <cellXfs count="57">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1268,26 +1384,20 @@
     <xf numFmtId="21" fontId="4" fillId="6" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="14" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="21" fontId="11" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1307,7 +1417,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Standard" xfId="0" builtinId="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -1570,37 +1680,37 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:F21"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="2" width="8" customWidth="1"/>
-    <col min="3" max="3" width="13.5546875" customWidth="1"/>
+    <col min="3" max="3" width="13.53125" customWidth="1"/>
     <col min="4" max="4" width="12" customWidth="1"/>
     <col min="5" max="5" width="14" customWidth="1"/>
-    <col min="6" max="6" width="22.77734375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="22.73046875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="46" t="s">
+    <row r="1" spans="1:6" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="48" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51"/>
-      <c r="E1" s="51"/>
-      <c r="F1" s="51"/>
-    </row>
-    <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="48" t="s">
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+    </row>
+    <row r="2" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="44" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="49"/>
-      <c r="C2" s="49"/>
-      <c r="D2" s="49"/>
-      <c r="E2" s="49"/>
-      <c r="F2" s="49"/>
-    </row>
-    <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="45"/>
+      <c r="C2" s="45"/>
+      <c r="D2" s="45"/>
+      <c r="E2" s="45"/>
+      <c r="F2" s="45"/>
+    </row>
+    <row r="3" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -1620,7 +1730,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="22" t="s">
         <v>8</v>
       </c>
@@ -1642,7 +1752,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="22" t="s">
         <v>10</v>
       </c>
@@ -1664,7 +1774,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="22" t="s">
         <v>11</v>
       </c>
@@ -1686,7 +1796,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="7" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="22" t="s">
         <v>12</v>
       </c>
@@ -1708,7 +1818,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="22" t="s">
         <v>13</v>
       </c>
@@ -1730,7 +1840,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="22" t="s">
         <v>14</v>
       </c>
@@ -1752,7 +1862,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="10" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="22" t="s">
         <v>15</v>
       </c>
@@ -1774,7 +1884,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="11" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="22" t="s">
         <v>16</v>
       </c>
@@ -1796,7 +1906,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="9" t="s">
         <v>8</v>
       </c>
@@ -1818,7 +1928,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="13" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="9" t="s">
         <v>10</v>
       </c>
@@ -1840,7 +1950,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="14" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="9" t="s">
         <v>14</v>
       </c>
@@ -1862,7 +1972,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="15" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" s="9" t="s">
         <v>15</v>
       </c>
@@ -1884,7 +1994,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="16" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A16" s="9" t="s">
         <v>16</v>
       </c>
@@ -1906,7 +2016,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="17" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" s="11" t="s">
         <v>8</v>
       </c>
@@ -1928,7 +2038,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="18" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A18" s="11" t="s">
         <v>14</v>
       </c>
@@ -1950,7 +2060,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="19" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A19" s="11" t="s">
         <v>15</v>
       </c>
@@ -1972,7 +2082,7 @@
         <v>915</v>
       </c>
     </row>
-    <row r="20" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" s="11" t="s">
         <v>16</v>
       </c>
@@ -1994,15 +2104,15 @@
         <v>915</v>
       </c>
     </row>
-    <row r="21" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A21" s="50" t="s">
+    <row r="21" spans="1:6" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A21" s="46" t="s">
         <v>19</v>
       </c>
-      <c r="B21" s="51"/>
-      <c r="C21" s="51"/>
-      <c r="D21" s="51"/>
-      <c r="E21" s="51"/>
-      <c r="F21" s="51"/>
+      <c r="B21" s="47"/>
+      <c r="C21" s="47"/>
+      <c r="D21" s="47"/>
+      <c r="E21" s="47"/>
+      <c r="F21" s="47"/>
     </row>
   </sheetData>
   <mergeCells count="3">
@@ -2017,21 +2127,21 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0900-000000000000}">
-  <dimension ref="A1:G23"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="9.109375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E34"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="15.21875" style="31" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="15.265625" style="31" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="16" style="31" customWidth="1"/>
     <col min="3" max="3" width="13" style="31" bestFit="1" customWidth="1"/>
-    <col min="4" max="16384" width="9.109375" style="31"/>
+    <col min="4" max="16384" width="9.06640625" style="31"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A1" s="35" t="s">
         <v>202</v>
       </c>
     </row>
-    <row r="2" spans="1:7" s="33" customFormat="1" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:5" s="33" customFormat="1" x14ac:dyDescent="0.4">
       <c r="A2" s="36" t="s">
         <v>213</v>
       </c>
@@ -2048,12 +2158,12 @@
         <v>230</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A3" s="37" t="s">
         <v>222</v>
       </c>
-      <c r="B3" s="45">
-        <v>0.25</v>
+      <c r="B3" s="37" t="s">
+        <v>231</v>
       </c>
       <c r="C3" s="38" t="s">
         <v>191</v>
@@ -2065,7 +2175,7 @@
         <v>232</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A4" s="37" t="s">
         <v>222</v>
       </c>
@@ -2073,78 +2183,75 @@
         <v>231</v>
       </c>
       <c r="C4" s="38" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="D4" s="39">
-        <v>3000</v>
+        <v>2600</v>
       </c>
       <c r="E4" s="37" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A5" s="37" t="s">
         <v>222</v>
       </c>
       <c r="B5" s="37" t="s">
-        <v>231</v>
+        <v>277</v>
       </c>
       <c r="C5" s="38" t="s">
-        <v>181</v>
+        <v>196</v>
       </c>
       <c r="D5" s="39">
-        <v>2600</v>
+        <v>3200</v>
       </c>
       <c r="E5" s="37" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A6" s="37" t="s">
         <v>222</v>
       </c>
       <c r="B6" s="37" t="s">
-        <v>231</v>
+        <v>278</v>
       </c>
       <c r="C6" s="38" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D6" s="39">
-        <v>2600</v>
+        <v>3000</v>
       </c>
       <c r="E6" s="37" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A7" s="37" t="s">
-        <v>222</v>
-      </c>
-      <c r="B7" s="45">
-        <v>0.53842592592592597</v>
+        <v>216</v>
+      </c>
+      <c r="B7" s="37" t="s">
+        <v>235</v>
       </c>
       <c r="C7" s="38" t="s">
-        <v>196</v>
+        <v>191</v>
       </c>
       <c r="D7" s="39">
-        <v>3200</v>
+        <v>1200</v>
       </c>
       <c r="E7" s="37" t="s">
-        <v>233</v>
-      </c>
-      <c r="G7" s="31" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A8" s="37" t="s">
-        <v>222</v>
-      </c>
-      <c r="B8" s="45">
-        <v>0.5556712962962963</v>
+        <v>216</v>
+      </c>
+      <c r="B8" s="37" t="s">
+        <v>236</v>
       </c>
       <c r="C8" s="38" t="s">
-        <v>161</v>
+        <v>191</v>
       </c>
       <c r="D8" s="39">
         <v>3000</v>
@@ -2152,269 +2259,447 @@
       <c r="E8" s="37" t="s">
         <v>234</v>
       </c>
-      <c r="G8" s="31" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A9" s="44">
-        <v>46266</v>
-      </c>
-      <c r="B9" s="45">
-        <v>0.60631944444444441</v>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A9" s="37" t="s">
+        <v>217</v>
+      </c>
+      <c r="B9" s="37" t="s">
+        <v>237</v>
       </c>
       <c r="C9" s="38" t="s">
+        <v>191</v>
+      </c>
+      <c r="D9" s="39">
+        <v>3000</v>
+      </c>
+      <c r="E9" s="37" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A10" s="37" t="s">
+        <v>217</v>
+      </c>
+      <c r="B10" s="37" t="s">
+        <v>238</v>
+      </c>
+      <c r="C10" s="38" t="s">
+        <v>181</v>
+      </c>
+      <c r="D10" s="39">
+        <v>2400</v>
+      </c>
+      <c r="E10" s="37" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="11" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A11" s="37" t="s">
+        <v>218</v>
+      </c>
+      <c r="B11" s="37" t="s">
+        <v>239</v>
+      </c>
+      <c r="C11" s="38" t="s">
         <v>169</v>
       </c>
-      <c r="D9" s="39">
-        <v>1200</v>
-      </c>
-      <c r="E9" s="37" t="s">
+      <c r="D11" s="39">
+        <v>2600</v>
+      </c>
+      <c r="E11" s="37" t="s">
         <v>234</v>
       </c>
-      <c r="G9" s="31" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A10" s="44">
-        <v>46266</v>
-      </c>
-      <c r="B10" s="45">
-        <v>0.68965277777777778</v>
-      </c>
-      <c r="C10" s="38" t="s">
-        <v>169</v>
-      </c>
-      <c r="D10" s="39">
-        <v>1200</v>
-      </c>
-      <c r="E10" s="37" t="s">
-        <v>232</v>
-      </c>
-      <c r="G10" s="31" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A11" s="37" t="s">
-        <v>216</v>
-      </c>
-      <c r="B11" s="37" t="s">
-        <v>235</v>
-      </c>
-      <c r="C11" s="38" t="s">
-        <v>191</v>
-      </c>
-      <c r="D11" s="39">
-        <v>1200</v>
-      </c>
-      <c r="E11" s="37" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+    </row>
+    <row r="12" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A12" s="37" t="s">
-        <v>216</v>
+        <v>218</v>
       </c>
       <c r="B12" s="37" t="s">
-        <v>236</v>
+        <v>240</v>
       </c>
       <c r="C12" s="38" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="D12" s="39">
-        <v>3000</v>
+        <v>1000</v>
       </c>
       <c r="E12" s="37" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A13" s="37" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="B13" s="37" t="s">
-        <v>237</v>
+        <v>241</v>
       </c>
       <c r="C13" s="38" t="s">
-        <v>191</v>
+        <v>181</v>
       </c>
       <c r="D13" s="39">
         <v>3000</v>
       </c>
       <c r="E13" s="37" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A14" s="37" t="s">
+        <v>218</v>
+      </c>
+      <c r="B14" s="37" t="s">
+        <v>242</v>
+      </c>
+      <c r="C14" s="38" t="s">
+        <v>169</v>
+      </c>
+      <c r="D14" s="39">
+        <v>2800</v>
+      </c>
+      <c r="E14" s="37" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A15" s="37" t="s">
+        <v>219</v>
+      </c>
+      <c r="B15" s="37" t="s">
+        <v>243</v>
+      </c>
+      <c r="C15" s="38" t="s">
+        <v>181</v>
+      </c>
+      <c r="D15" s="39">
+        <v>1600</v>
+      </c>
+      <c r="E15" s="37" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A16" s="37" t="s">
+        <v>220</v>
+      </c>
+      <c r="B16" s="37" t="s">
+        <v>244</v>
+      </c>
+      <c r="C16" s="38" t="s">
+        <v>191</v>
+      </c>
+      <c r="D16" s="39">
+        <v>1400</v>
+      </c>
+      <c r="E16" s="37" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A14" s="37" t="s">
-        <v>217</v>
-      </c>
-      <c r="B14" s="37" t="s">
-        <v>238</v>
-      </c>
-      <c r="C14" s="38" t="s">
-        <v>181</v>
-      </c>
-      <c r="D14" s="39">
-        <v>2400</v>
-      </c>
-      <c r="E14" s="37" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A15" s="37" t="s">
-        <v>218</v>
-      </c>
-      <c r="B15" s="37" t="s">
-        <v>239</v>
-      </c>
-      <c r="C15" s="38" t="s">
-        <v>169</v>
-      </c>
-      <c r="D15" s="39">
-        <v>2600</v>
-      </c>
-      <c r="E15" s="37" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A16" s="37" t="s">
-        <v>218</v>
-      </c>
-      <c r="B16" s="37" t="s">
-        <v>240</v>
-      </c>
-      <c r="C16" s="38" t="s">
-        <v>181</v>
-      </c>
-      <c r="D16" s="39">
-        <v>1000</v>
-      </c>
-      <c r="E16" s="37" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A17" s="37" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B17" s="37" t="s">
-        <v>241</v>
+        <v>245</v>
       </c>
       <c r="C17" s="38" t="s">
-        <v>181</v>
+        <v>191</v>
       </c>
       <c r="D17" s="39">
+        <v>3600</v>
+      </c>
+      <c r="E17" s="37" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A18" s="37" t="s">
+        <v>220</v>
+      </c>
+      <c r="B18" s="37" t="s">
+        <v>246</v>
+      </c>
+      <c r="C18" s="38" t="s">
+        <v>161</v>
+      </c>
+      <c r="D18" s="39">
         <v>3000</v>
-      </c>
-      <c r="E17" s="37" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" s="37" t="s">
-        <v>218</v>
-      </c>
-      <c r="B18" s="37" t="s">
-        <v>242</v>
-      </c>
-      <c r="C18" s="38" t="s">
-        <v>169</v>
-      </c>
-      <c r="D18" s="39">
-        <v>2800</v>
       </c>
       <c r="E18" s="37" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A19" s="37" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B19" s="37" t="s">
-        <v>243</v>
+        <v>247</v>
       </c>
       <c r="C19" s="38" t="s">
-        <v>181</v>
+        <v>161</v>
       </c>
       <c r="D19" s="39">
         <v>1600</v>
       </c>
       <c r="E19" s="37" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.35">
       <c r="A20" s="37" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B20" s="37" t="s">
-        <v>244</v>
+        <v>308</v>
       </c>
       <c r="C20" s="38" t="s">
         <v>191</v>
       </c>
       <c r="D20" s="39">
-        <v>1400</v>
+        <v>5000</v>
       </c>
       <c r="E20" s="37" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A21" s="37" t="s">
+        <v>221</v>
+      </c>
+      <c r="B21" s="37" t="s">
+        <v>309</v>
+      </c>
+      <c r="C21" s="38" t="s">
+        <v>181</v>
+      </c>
+      <c r="D21" s="39">
+        <v>2000</v>
+      </c>
+      <c r="E21" s="37" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A22" s="37" t="s">
+        <v>282</v>
+      </c>
+      <c r="B22" s="37" t="s">
+        <v>310</v>
+      </c>
+      <c r="C22" s="38" t="s">
+        <v>181</v>
+      </c>
+      <c r="D22" s="39">
+        <v>3400</v>
+      </c>
+      <c r="E22" s="37" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A23" s="37" t="s">
+        <v>282</v>
+      </c>
+      <c r="B23" s="37" t="s">
+        <v>311</v>
+      </c>
+      <c r="C23" s="38" t="s">
+        <v>191</v>
+      </c>
+      <c r="D23" s="39">
+        <v>3400</v>
+      </c>
+      <c r="E23" s="37" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" s="37" t="s">
-        <v>220</v>
-      </c>
-      <c r="B21" s="37" t="s">
-        <v>245</v>
-      </c>
-      <c r="C21" s="38" t="s">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A24" s="37" t="s">
+        <v>287</v>
+      </c>
+      <c r="B24" s="37" t="s">
+        <v>312</v>
+      </c>
+      <c r="C24" s="38" t="s">
+        <v>181</v>
+      </c>
+      <c r="D24" s="39">
+        <v>1600</v>
+      </c>
+      <c r="E24" s="37" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A25" s="37" t="s">
+        <v>287</v>
+      </c>
+      <c r="B25" s="37" t="s">
+        <v>313</v>
+      </c>
+      <c r="C25" s="38" t="s">
+        <v>161</v>
+      </c>
+      <c r="D25" s="39">
+        <v>3000</v>
+      </c>
+      <c r="E25" s="37" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A26" s="37" t="s">
+        <v>287</v>
+      </c>
+      <c r="B26" s="37" t="s">
+        <v>314</v>
+      </c>
+      <c r="C26" s="38" t="s">
+        <v>181</v>
+      </c>
+      <c r="D26" s="39">
+        <v>2000</v>
+      </c>
+      <c r="E26" s="37" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A27" s="37" t="s">
+        <v>291</v>
+      </c>
+      <c r="B27" s="37" t="s">
+        <v>315</v>
+      </c>
+      <c r="C27" s="38" t="s">
+        <v>181</v>
+      </c>
+      <c r="D27" s="39">
+        <v>800</v>
+      </c>
+      <c r="E27" s="37" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A28" s="37" t="s">
+        <v>291</v>
+      </c>
+      <c r="B28" s="37" t="s">
+        <v>316</v>
+      </c>
+      <c r="C28" s="38" t="s">
+        <v>196</v>
+      </c>
+      <c r="D28" s="39">
+        <v>2800</v>
+      </c>
+      <c r="E28" s="37" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A29" s="37" t="s">
+        <v>291</v>
+      </c>
+      <c r="B29" s="37" t="s">
+        <v>317</v>
+      </c>
+      <c r="C29" s="38" t="s">
         <v>191</v>
       </c>
-      <c r="D21" s="39">
-        <v>3600</v>
-      </c>
-      <c r="E21" s="37" t="s">
+      <c r="D29" s="39">
+        <v>3000</v>
+      </c>
+      <c r="E29" s="37" t="s">
         <v>232</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" s="37" t="s">
-        <v>220</v>
-      </c>
-      <c r="B22" s="37" t="s">
-        <v>246</v>
-      </c>
-      <c r="C22" s="38" t="s">
-        <v>161</v>
-      </c>
-      <c r="D22" s="39">
+    <row r="30" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A30" s="37" t="s">
+        <v>291</v>
+      </c>
+      <c r="B30" s="37" t="s">
+        <v>318</v>
+      </c>
+      <c r="C30" s="38" t="s">
+        <v>191</v>
+      </c>
+      <c r="D30" s="39">
         <v>3000</v>
       </c>
-      <c r="E22" s="37" t="s">
+      <c r="E30" s="37" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" s="37" t="s">
-        <v>221</v>
-      </c>
-      <c r="B23" s="37" t="s">
-        <v>247</v>
-      </c>
-      <c r="C23" s="38" t="s">
-        <v>161</v>
-      </c>
-      <c r="D23" s="39">
-        <v>1600</v>
-      </c>
-      <c r="E23" s="37" t="s">
+    <row r="31" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A31" s="37" t="s">
+        <v>297</v>
+      </c>
+      <c r="B31" s="37" t="s">
+        <v>319</v>
+      </c>
+      <c r="C31" s="38" t="s">
+        <v>181</v>
+      </c>
+      <c r="D31" s="39">
+        <v>3400</v>
+      </c>
+      <c r="E31" s="37" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A32" s="37" t="s">
+        <v>302</v>
+      </c>
+      <c r="B32" s="37" t="s">
+        <v>320</v>
+      </c>
+      <c r="C32" s="38" t="s">
+        <v>196</v>
+      </c>
+      <c r="D32" s="39">
+        <v>200</v>
+      </c>
+      <c r="E32" s="37" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A33" s="37" t="s">
+        <v>302</v>
+      </c>
+      <c r="B33" s="37" t="s">
+        <v>321</v>
+      </c>
+      <c r="C33" s="38" t="s">
+        <v>191</v>
+      </c>
+      <c r="D33" s="39">
+        <v>4000</v>
+      </c>
+      <c r="E33" s="37" t="s">
         <v>234</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.35">
+      <c r="A34" s="37" t="s">
+        <v>302</v>
+      </c>
+      <c r="B34" s="37" t="s">
+        <v>322</v>
+      </c>
+      <c r="C34" s="38" t="s">
+        <v>181</v>
+      </c>
+      <c r="D34" s="39">
+        <v>4000</v>
+      </c>
+      <c r="E34" s="37" t="s">
+        <v>233</v>
       </c>
     </row>
   </sheetData>
@@ -2425,16 +2710,16 @@
 <file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0800-000000000000}">
   <dimension ref="A1:I64"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="16" style="21" customWidth="1"/>
     <col min="2" max="2" width="12" style="21" customWidth="1"/>
     <col min="3" max="3" width="16" style="21" customWidth="1"/>
-    <col min="4" max="6" width="5.77734375" style="31" customWidth="1"/>
-    <col min="8" max="8" width="119.5546875" customWidth="1"/>
+    <col min="4" max="6" width="5.796875" style="31" customWidth="1"/>
+    <col min="8" max="8" width="119.59765625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:9" ht="28.5" x14ac:dyDescent="0.45">
       <c r="A1" s="32" t="s">
         <v>145</v>
       </c>
@@ -2458,7 +2743,7 @@
       </c>
       <c r="I1" s="30"/>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A2" s="21" t="s">
         <v>84</v>
       </c>
@@ -2473,7 +2758,7 @@
       </c>
       <c r="H2" s="25"/>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A3" s="21" t="s">
         <v>86</v>
       </c>
@@ -2487,7 +2772,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A4" s="21" t="s">
         <v>89</v>
       </c>
@@ -2501,7 +2786,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A5" s="21" t="s">
         <v>88</v>
       </c>
@@ -2515,7 +2800,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A6" s="21" t="s">
         <v>91</v>
       </c>
@@ -2529,7 +2814,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A7" s="21" t="s">
         <v>90</v>
       </c>
@@ -2543,7 +2828,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A8" s="21" t="s">
         <v>148</v>
       </c>
@@ -2560,7 +2845,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A9" s="21" t="s">
         <v>149</v>
       </c>
@@ -2577,7 +2862,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A10" s="21" t="s">
         <v>150</v>
       </c>
@@ -2591,7 +2876,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A11" s="21" t="s">
         <v>151</v>
       </c>
@@ -2608,7 +2893,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A12" s="21" t="s">
         <v>152</v>
       </c>
@@ -2622,7 +2907,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A13" s="21" t="s">
         <v>153</v>
       </c>
@@ -2639,7 +2924,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A14" s="21" t="s">
         <v>154</v>
       </c>
@@ -2653,7 +2938,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A15" s="21" t="s">
         <v>155</v>
       </c>
@@ -2667,7 +2952,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.45">
       <c r="A16" s="21" t="s">
         <v>156</v>
       </c>
@@ -2681,7 +2966,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A17" s="21" t="s">
         <v>157</v>
       </c>
@@ -2695,7 +2980,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A18" s="21" t="s">
         <v>158</v>
       </c>
@@ -2709,7 +2994,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A19" s="21" t="s">
         <v>85</v>
       </c>
@@ -2729,7 +3014,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A20" s="21" t="s">
         <v>159</v>
       </c>
@@ -2743,7 +3028,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A21" s="21" t="s">
         <v>160</v>
       </c>
@@ -2757,7 +3042,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A22" s="21" t="s">
         <v>161</v>
       </c>
@@ -2777,7 +3062,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A23" s="21" t="s">
         <v>162</v>
       </c>
@@ -2791,7 +3076,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A24" s="21" t="s">
         <v>163</v>
       </c>
@@ -2805,7 +3090,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A25" s="21" t="s">
         <v>164</v>
       </c>
@@ -2819,7 +3104,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A26" s="21" t="s">
         <v>165</v>
       </c>
@@ -2833,7 +3118,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A27" s="21" t="s">
         <v>166</v>
       </c>
@@ -2847,7 +3132,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A28" s="21" t="s">
         <v>167</v>
       </c>
@@ -2861,7 +3146,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A29" s="21" t="s">
         <v>168</v>
       </c>
@@ -2878,7 +3163,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A30" s="21" t="s">
         <v>169</v>
       </c>
@@ -2892,7 +3177,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A31" s="21" t="s">
         <v>170</v>
       </c>
@@ -2906,7 +3191,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A32" s="21" t="s">
         <v>171</v>
       </c>
@@ -2920,7 +3205,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A33" s="21" t="s">
         <v>172</v>
       </c>
@@ -2937,7 +3222,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A34" s="21" t="s">
         <v>173</v>
       </c>
@@ -2954,7 +3239,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A35" s="21" t="s">
         <v>174</v>
       </c>
@@ -2974,7 +3259,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A36" s="21" t="s">
         <v>175</v>
       </c>
@@ -2991,7 +3276,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A37" s="21" t="s">
         <v>176</v>
       </c>
@@ -3008,7 +3293,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A38" s="21" t="s">
         <v>177</v>
       </c>
@@ -3025,7 +3310,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A39" s="21" t="s">
         <v>178</v>
       </c>
@@ -3042,7 +3327,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A40" s="21" t="s">
         <v>179</v>
       </c>
@@ -3059,7 +3344,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A41" s="21" t="s">
         <v>180</v>
       </c>
@@ -3076,7 +3361,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A42" s="21" t="s">
         <v>181</v>
       </c>
@@ -3093,7 +3378,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A43" s="21" t="s">
         <v>182</v>
       </c>
@@ -3110,7 +3395,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A44" s="21" t="s">
         <v>183</v>
       </c>
@@ -3127,7 +3412,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A45" s="21" t="s">
         <v>184</v>
       </c>
@@ -3144,7 +3429,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A46" s="21" t="s">
         <v>185</v>
       </c>
@@ -3161,7 +3446,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A47" s="21" t="s">
         <v>186</v>
       </c>
@@ -3178,7 +3463,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A48" s="21" t="s">
         <v>187</v>
       </c>
@@ -3195,7 +3480,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A49" s="21" t="s">
         <v>188</v>
       </c>
@@ -3212,7 +3497,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A50" s="21" t="s">
         <v>189</v>
       </c>
@@ -3229,7 +3514,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A51" s="21" t="s">
         <v>190</v>
       </c>
@@ -3246,7 +3531,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A52" s="21" t="s">
         <v>191</v>
       </c>
@@ -3263,7 +3548,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A53" s="21" t="s">
         <v>192</v>
       </c>
@@ -3280,7 +3565,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A54" s="21" t="s">
         <v>193</v>
       </c>
@@ -3294,7 +3579,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A55" s="21" t="s">
         <v>194</v>
       </c>
@@ -3311,7 +3596,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A56" s="21" t="s">
         <v>195</v>
       </c>
@@ -3325,7 +3610,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A57" s="21" t="s">
         <v>196</v>
       </c>
@@ -3342,7 +3627,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A58" s="21" t="s">
         <v>197</v>
       </c>
@@ -3359,7 +3644,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A59" s="21" t="s">
         <v>198</v>
       </c>
@@ -3376,7 +3661,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A60" s="21" t="s">
         <v>92</v>
       </c>
@@ -3393,7 +3678,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A61" s="21" t="s">
         <v>199</v>
       </c>
@@ -3410,7 +3695,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A62" s="21" t="s">
         <v>200</v>
       </c>
@@ -3427,7 +3712,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A63" s="21" t="s">
         <v>201</v>
       </c>
@@ -3444,7 +3729,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A64" s="21" t="s">
         <v>93</v>
       </c>
@@ -3466,13 +3751,13 @@
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{13E7B77F-25BE-4F53-8466-968392D830E1}">
   <dimension ref="A1:C4"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="24.33203125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="12.21875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="12.265625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A1" s="1" t="s">
         <v>96</v>
       </c>
@@ -3483,7 +3768,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A2" s="32" t="s">
         <v>210</v>
       </c>
@@ -3494,7 +3779,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A3" s="32" t="s">
         <v>208</v>
       </c>
@@ -3505,7 +3790,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" x14ac:dyDescent="0.45">
       <c r="A4" s="32" t="s">
         <v>214</v>
       </c>
@@ -3524,7 +3809,7 @@
 <file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0A00-000000000000}">
   <dimension ref="A1:F8"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="10" customWidth="1"/>
     <col min="2" max="2" width="16" customWidth="1"/>
@@ -3533,7 +3818,7 @@
     <col min="6" max="6" width="90" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A1" s="29" t="s">
         <v>3</v>
       </c>
@@ -3550,7 +3835,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -3564,7 +3849,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -3578,7 +3863,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -3592,7 +3877,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>17</v>
       </c>
@@ -3606,7 +3891,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>17</v>
       </c>
@@ -3620,7 +3905,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>18</v>
       </c>
@@ -3634,7 +3919,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>18</v>
       </c>
@@ -3656,20 +3941,20 @@
 <file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0700-000000000000}">
   <dimension ref="A1:C18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
     <col min="2" max="3" width="60" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="46" t="s">
+    <row r="1" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="48" t="s">
         <v>112</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
-    </row>
-    <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+    </row>
+    <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>113</v>
       </c>
@@ -3680,7 +3965,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="20" t="s">
         <v>116</v>
       </c>
@@ -3691,7 +3976,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="4" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="17" t="s">
         <v>119</v>
       </c>
@@ -3702,7 +3987,7 @@
         <v>121</v>
       </c>
     </row>
-    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="20" t="s">
         <v>122</v>
       </c>
@@ -3713,7 +3998,7 @@
         <v>124</v>
       </c>
     </row>
-    <row r="6" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="17" t="s">
         <v>125</v>
       </c>
@@ -3724,7 +4009,7 @@
         <v>127</v>
       </c>
     </row>
-    <row r="7" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="20" t="s">
         <v>128</v>
       </c>
@@ -3735,7 +4020,7 @@
         <v>130</v>
       </c>
     </row>
-    <row r="8" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="17" t="s">
         <v>131</v>
       </c>
@@ -3746,7 +4031,7 @@
         <v>133</v>
       </c>
     </row>
-    <row r="9" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="20" t="s">
         <v>134</v>
       </c>
@@ -3757,7 +4042,7 @@
         <v>136</v>
       </c>
     </row>
-    <row r="10" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="17" t="s">
         <v>137</v>
       </c>
@@ -3766,48 +4051,48 @@
       </c>
       <c r="C10" s="14"/>
     </row>
-    <row r="11" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.3"/>
-    <row r="13" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="48" t="s">
+    <row r="11" spans="1:3" ht="39.75" customHeight="1" x14ac:dyDescent="0.45"/>
+    <row r="13" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A13" s="44" t="s">
         <v>139</v>
       </c>
-      <c r="B13" s="49"/>
-      <c r="C13" s="49"/>
-    </row>
-    <row r="14" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="53" t="s">
+      <c r="B13" s="45"/>
+      <c r="C13" s="45"/>
+    </row>
+    <row r="14" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A14" s="51" t="s">
         <v>140</v>
       </c>
-      <c r="B14" s="49"/>
-      <c r="C14" s="54"/>
-    </row>
-    <row r="15" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A15" s="57" t="s">
+      <c r="B14" s="45"/>
+      <c r="C14" s="52"/>
+    </row>
+    <row r="15" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A15" s="55" t="s">
         <v>141</v>
       </c>
-      <c r="B15" s="49"/>
-      <c r="C15" s="54"/>
-    </row>
-    <row r="16" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="58" t="s">
+      <c r="B15" s="45"/>
+      <c r="C15" s="52"/>
+    </row>
+    <row r="16" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A16" s="56" t="s">
         <v>142</v>
       </c>
-      <c r="B16" s="49"/>
-      <c r="C16" s="54"/>
-    </row>
-    <row r="17" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A17" s="55" t="s">
+      <c r="B16" s="45"/>
+      <c r="C16" s="52"/>
+    </row>
+    <row r="17" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A17" s="53" t="s">
         <v>143</v>
       </c>
-      <c r="B17" s="49"/>
-      <c r="C17" s="54"/>
-    </row>
-    <row r="18" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A18" s="56" t="s">
+      <c r="B17" s="45"/>
+      <c r="C17" s="52"/>
+    </row>
+    <row r="18" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A18" s="54" t="s">
         <v>144</v>
       </c>
-      <c r="B18" s="49"/>
-      <c r="C18" s="54"/>
+      <c r="B18" s="45"/>
+      <c r="C18" s="52"/>
     </row>
   </sheetData>
   <mergeCells count="7">
@@ -3827,36 +4112,36 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E21CF094-4655-472A-BF18-B41A224CE48A}">
   <dimension ref="A1:F54"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="2" max="2" width="10.109375" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="11.88671875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="9.796875" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="11.9296875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" ht="16.8" x14ac:dyDescent="0.3">
-      <c r="A1" s="46" t="s">
-        <v>262</v>
-      </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51"/>
-      <c r="E1" s="51"/>
-      <c r="F1" s="51"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" ht="16.899999999999999" x14ac:dyDescent="0.45">
+      <c r="A1" s="48" t="s">
+        <v>261</v>
+      </c>
+      <c r="B1" s="48"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
-        <v>262</v>
+        <v>261</v>
       </c>
       <c r="B2" s="1" t="s">
+        <v>274</v>
+      </c>
+      <c r="C2" s="1" t="s">
         <v>275</v>
       </c>
-      <c r="C2" s="1" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A3" s="6" t="s">
-        <v>264</v>
+        <v>263</v>
       </c>
       <c r="B3" s="43">
         <v>0.25</v>
@@ -3865,9 +4150,9 @@
         <v>0.58332175925925922</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A4" s="6" t="s">
-        <v>265</v>
+        <v>264</v>
       </c>
       <c r="B4" s="43">
         <v>0.58333333333333337</v>
@@ -3876,9 +4161,9 @@
         <v>0.91665509259259259</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A5" s="6" t="s">
-        <v>266</v>
+        <v>265</v>
       </c>
       <c r="B5" s="43">
         <v>0.91666666666666663</v>
@@ -3887,27 +4172,27 @@
         <v>0.24998842592592593</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A6" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B6" s="1" t="s">
+        <v>262</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>273</v>
+      </c>
+      <c r="D6" s="1" t="s">
         <v>263</v>
       </c>
-      <c r="C6" s="1" t="s">
-        <v>274</v>
-      </c>
-      <c r="D6" s="1" t="s">
+      <c r="E6" s="1" t="s">
         <v>264</v>
       </c>
-      <c r="E6" s="1" t="s">
+      <c r="F6" s="1" t="s">
         <v>265</v>
       </c>
-      <c r="F6" s="1" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A7" s="6" t="s">
         <v>9</v>
       </c>
@@ -3915,7 +4200,7 @@
         <v>46266</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D7" s="3" t="s">
         <v>211</v>
@@ -3927,7 +4212,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A8" s="6" t="s">
         <v>9</v>
       </c>
@@ -3935,7 +4220,7 @@
         <v>46267</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D8" s="3" t="s">
         <v>211</v>
@@ -3947,7 +4232,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A9" s="6" t="s">
         <v>9</v>
       </c>
@@ -3955,7 +4240,7 @@
         <v>46268</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D9" s="3" t="s">
         <v>211</v>
@@ -3967,7 +4252,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A10" s="6" t="s">
         <v>9</v>
       </c>
@@ -3975,7 +4260,7 @@
         <v>46269</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D10" s="3" t="s">
         <v>211</v>
@@ -3987,7 +4272,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A11" s="6" t="s">
         <v>9</v>
       </c>
@@ -3995,19 +4280,15 @@
         <v>46270</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D11" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="E11" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="F11" s="3" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E11" s="3"/>
+      <c r="F11" s="3"/>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A12" s="6" t="s">
         <v>9</v>
       </c>
@@ -4015,13 +4296,13 @@
         <v>46271</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D12" s="3"/>
       <c r="E12" s="3"/>
       <c r="F12" s="3"/>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A13" s="6" t="s">
         <v>9</v>
       </c>
@@ -4029,7 +4310,7 @@
         <v>46272</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D13" s="3" t="s">
         <v>211</v>
@@ -4041,7 +4322,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A14" s="6" t="s">
         <v>9</v>
       </c>
@@ -4049,13 +4330,19 @@
         <v>46273</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="D14" s="3"/>
-      <c r="E14" s="3"/>
-      <c r="F14" s="3"/>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+        <v>267</v>
+      </c>
+      <c r="D14" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E14" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="F14" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A15" s="6" t="s">
         <v>9</v>
       </c>
@@ -4063,13 +4350,19 @@
         <v>46274</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>269</v>
-      </c>
-      <c r="D15" s="3"/>
-      <c r="E15" s="3"/>
-      <c r="F15" s="3"/>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+        <v>268</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E15" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="F15" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A16" s="6" t="s">
         <v>9</v>
       </c>
@@ -4077,13 +4370,19 @@
         <v>46275</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>270</v>
-      </c>
-      <c r="D16" s="3"/>
-      <c r="E16" s="3"/>
-      <c r="F16" s="3"/>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+        <v>269</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E16" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="F16" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A17" s="6" t="s">
         <v>9</v>
       </c>
@@ -4091,13 +4390,19 @@
         <v>46276</v>
       </c>
       <c r="C17" s="6" t="s">
-        <v>271</v>
-      </c>
-      <c r="D17" s="3"/>
-      <c r="E17" s="3"/>
-      <c r="F17" s="3"/>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+        <v>270</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E17" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="F17" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A18" s="6" t="s">
         <v>9</v>
       </c>
@@ -4105,13 +4410,15 @@
         <v>46277</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>272</v>
-      </c>
-      <c r="D18" s="3"/>
+        <v>271</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>211</v>
+      </c>
       <c r="E18" s="3"/>
       <c r="F18" s="3"/>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A19" s="6" t="s">
         <v>9</v>
       </c>
@@ -4119,13 +4426,13 @@
         <v>46278</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D19" s="3"/>
       <c r="E19" s="3"/>
       <c r="F19" s="3"/>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A20" s="6" t="s">
         <v>9</v>
       </c>
@@ -4133,13 +4440,19 @@
         <v>46279</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>267</v>
-      </c>
-      <c r="D20" s="3"/>
-      <c r="E20" s="3"/>
-      <c r="F20" s="3"/>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+        <v>266</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E20" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="F20" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A21" s="6" t="s">
         <v>9</v>
       </c>
@@ -4147,13 +4460,19 @@
         <v>46280</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>268</v>
-      </c>
-      <c r="D21" s="3"/>
-      <c r="E21" s="3"/>
-      <c r="F21" s="3"/>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+        <v>267</v>
+      </c>
+      <c r="D21" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E21" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="F21" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A22" s="6" t="s">
         <v>9</v>
       </c>
@@ -4161,13 +4480,19 @@
         <v>46281</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>269</v>
-      </c>
-      <c r="D22" s="3"/>
-      <c r="E22" s="3"/>
-      <c r="F22" s="3"/>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+        <v>268</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E22" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="F22" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A23" s="10" t="s">
         <v>17</v>
       </c>
@@ -4175,7 +4500,7 @@
         <v>46266</v>
       </c>
       <c r="C23" s="10" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D23" s="3" t="s">
         <v>211</v>
@@ -4187,7 +4512,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A24" s="10" t="s">
         <v>17</v>
       </c>
@@ -4195,7 +4520,7 @@
         <v>46267</v>
       </c>
       <c r="C24" s="10" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>211</v>
@@ -4207,7 +4532,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A25" s="10" t="s">
         <v>17</v>
       </c>
@@ -4215,7 +4540,7 @@
         <v>46268</v>
       </c>
       <c r="C25" s="10" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>211</v>
@@ -4227,7 +4552,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A26" s="10" t="s">
         <v>17</v>
       </c>
@@ -4235,7 +4560,7 @@
         <v>46269</v>
       </c>
       <c r="C26" s="10" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>211</v>
@@ -4247,7 +4572,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A27" s="10" t="s">
         <v>17</v>
       </c>
@@ -4255,19 +4580,15 @@
         <v>46270</v>
       </c>
       <c r="C27" s="10" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="E27" s="3" t="s">
-        <v>211</v>
-      </c>
-      <c r="F27" s="3" t="s">
-        <v>211</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="E27" s="3"/>
+      <c r="F27" s="3"/>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A28" s="10" t="s">
         <v>17</v>
       </c>
@@ -4275,13 +4596,13 @@
         <v>46271</v>
       </c>
       <c r="C28" s="10" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D28" s="3"/>
       <c r="E28" s="3"/>
       <c r="F28" s="3"/>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A29" s="10" t="s">
         <v>17</v>
       </c>
@@ -4289,7 +4610,7 @@
         <v>46272</v>
       </c>
       <c r="C29" s="10" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>211</v>
@@ -4301,7 +4622,7 @@
         <v>211</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A30" s="10" t="s">
         <v>17</v>
       </c>
@@ -4309,13 +4630,19 @@
         <v>46273</v>
       </c>
       <c r="C30" s="10" t="s">
-        <v>268</v>
-      </c>
-      <c r="D30" s="3"/>
-      <c r="E30" s="3"/>
-      <c r="F30" s="3"/>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+        <v>267</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E30" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="F30" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A31" s="10" t="s">
         <v>17</v>
       </c>
@@ -4323,13 +4650,19 @@
         <v>46274</v>
       </c>
       <c r="C31" s="10" t="s">
-        <v>269</v>
-      </c>
-      <c r="D31" s="3"/>
-      <c r="E31" s="3"/>
-      <c r="F31" s="3"/>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+        <v>268</v>
+      </c>
+      <c r="D31" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E31" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="F31" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A32" s="10" t="s">
         <v>17</v>
       </c>
@@ -4337,13 +4670,19 @@
         <v>46275</v>
       </c>
       <c r="C32" s="10" t="s">
-        <v>270</v>
-      </c>
-      <c r="D32" s="3"/>
-      <c r="E32" s="3"/>
-      <c r="F32" s="3"/>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+        <v>269</v>
+      </c>
+      <c r="D32" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E32" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="F32" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A33" s="10" t="s">
         <v>17</v>
       </c>
@@ -4351,13 +4690,19 @@
         <v>46276</v>
       </c>
       <c r="C33" s="10" t="s">
-        <v>271</v>
-      </c>
-      <c r="D33" s="3"/>
-      <c r="E33" s="3"/>
-      <c r="F33" s="3"/>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+        <v>270</v>
+      </c>
+      <c r="D33" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E33" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="F33" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A34" s="10" t="s">
         <v>17</v>
       </c>
@@ -4365,13 +4710,15 @@
         <v>46277</v>
       </c>
       <c r="C34" s="10" t="s">
-        <v>272</v>
-      </c>
-      <c r="D34" s="3"/>
+        <v>271</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>211</v>
+      </c>
       <c r="E34" s="3"/>
       <c r="F34" s="3"/>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A35" s="10" t="s">
         <v>17</v>
       </c>
@@ -4379,13 +4726,13 @@
         <v>46278</v>
       </c>
       <c r="C35" s="10" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D35" s="3"/>
       <c r="E35" s="3"/>
       <c r="F35" s="3"/>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A36" s="10" t="s">
         <v>17</v>
       </c>
@@ -4393,13 +4740,19 @@
         <v>46279</v>
       </c>
       <c r="C36" s="10" t="s">
-        <v>267</v>
-      </c>
-      <c r="D36" s="3"/>
-      <c r="E36" s="3"/>
-      <c r="F36" s="3"/>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+        <v>266</v>
+      </c>
+      <c r="D36" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E36" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="F36" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A37" s="10" t="s">
         <v>17</v>
       </c>
@@ -4407,13 +4760,19 @@
         <v>46280</v>
       </c>
       <c r="C37" s="10" t="s">
-        <v>268</v>
-      </c>
-      <c r="D37" s="3"/>
-      <c r="E37" s="3"/>
-      <c r="F37" s="3"/>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+        <v>267</v>
+      </c>
+      <c r="D37" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E37" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="F37" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A38" s="10" t="s">
         <v>17</v>
       </c>
@@ -4421,13 +4780,19 @@
         <v>46281</v>
       </c>
       <c r="C38" s="10" t="s">
-        <v>269</v>
-      </c>
-      <c r="D38" s="3"/>
-      <c r="E38" s="3"/>
-      <c r="F38" s="3"/>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+        <v>268</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E38" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="F38" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A39" s="12" t="s">
         <v>18</v>
       </c>
@@ -4435,7 +4800,7 @@
         <v>46266</v>
       </c>
       <c r="C39" s="12" t="s">
-        <v>268</v>
+        <v>267</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>211</v>
@@ -4443,9 +4808,11 @@
       <c r="E39" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="F39" s="3"/>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F39" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A40" s="12" t="s">
         <v>18</v>
       </c>
@@ -4453,7 +4820,7 @@
         <v>46267</v>
       </c>
       <c r="C40" s="12" t="s">
-        <v>269</v>
+        <v>268</v>
       </c>
       <c r="D40" s="3" t="s">
         <v>211</v>
@@ -4461,9 +4828,11 @@
       <c r="E40" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="F40" s="3"/>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F40" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A41" s="12" t="s">
         <v>18</v>
       </c>
@@ -4471,7 +4840,7 @@
         <v>46268</v>
       </c>
       <c r="C41" s="12" t="s">
-        <v>270</v>
+        <v>269</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>211</v>
@@ -4479,9 +4848,11 @@
       <c r="E41" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="F41" s="3"/>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F41" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A42" s="12" t="s">
         <v>18</v>
       </c>
@@ -4489,7 +4860,7 @@
         <v>46269</v>
       </c>
       <c r="C42" s="12" t="s">
-        <v>271</v>
+        <v>270</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>211</v>
@@ -4497,9 +4868,11 @@
       <c r="E42" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="F42" s="3"/>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F42" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A43" s="12" t="s">
         <v>18</v>
       </c>
@@ -4507,17 +4880,15 @@
         <v>46270</v>
       </c>
       <c r="C43" s="12" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="E43" s="3" t="s">
-        <v>211</v>
-      </c>
+      <c r="E43" s="3"/>
       <c r="F43" s="3"/>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A44" s="12" t="s">
         <v>18</v>
       </c>
@@ -4525,13 +4896,13 @@
         <v>46271</v>
       </c>
       <c r="C44" s="12" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D44" s="3"/>
       <c r="E44" s="3"/>
       <c r="F44" s="3"/>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A45" s="12" t="s">
         <v>18</v>
       </c>
@@ -4539,7 +4910,7 @@
         <v>46272</v>
       </c>
       <c r="C45" s="12" t="s">
-        <v>267</v>
+        <v>266</v>
       </c>
       <c r="D45" s="3" t="s">
         <v>211</v>
@@ -4547,9 +4918,11 @@
       <c r="E45" s="3" t="s">
         <v>211</v>
       </c>
-      <c r="F45" s="3"/>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="F45" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A46" s="12" t="s">
         <v>18</v>
       </c>
@@ -4557,13 +4930,19 @@
         <v>46273</v>
       </c>
       <c r="C46" s="12" t="s">
-        <v>268</v>
-      </c>
-      <c r="D46" s="3"/>
-      <c r="E46" s="3"/>
-      <c r="F46" s="3"/>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+        <v>267</v>
+      </c>
+      <c r="D46" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E46" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="F46" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A47" s="12" t="s">
         <v>18</v>
       </c>
@@ -4571,13 +4950,19 @@
         <v>46274</v>
       </c>
       <c r="C47" s="12" t="s">
-        <v>269</v>
-      </c>
-      <c r="D47" s="3"/>
-      <c r="E47" s="3"/>
-      <c r="F47" s="3"/>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+        <v>268</v>
+      </c>
+      <c r="D47" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E47" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="F47" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A48" s="12" t="s">
         <v>18</v>
       </c>
@@ -4585,13 +4970,19 @@
         <v>46275</v>
       </c>
       <c r="C48" s="12" t="s">
-        <v>270</v>
-      </c>
-      <c r="D48" s="3"/>
-      <c r="E48" s="3"/>
-      <c r="F48" s="3"/>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+        <v>269</v>
+      </c>
+      <c r="D48" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E48" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="F48" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A49" s="12" t="s">
         <v>18</v>
       </c>
@@ -4599,13 +4990,19 @@
         <v>46276</v>
       </c>
       <c r="C49" s="12" t="s">
-        <v>271</v>
-      </c>
-      <c r="D49" s="3"/>
-      <c r="E49" s="3"/>
-      <c r="F49" s="3"/>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+        <v>270</v>
+      </c>
+      <c r="D49" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E49" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="F49" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A50" s="12" t="s">
         <v>18</v>
       </c>
@@ -4613,13 +5010,15 @@
         <v>46277</v>
       </c>
       <c r="C50" s="12" t="s">
-        <v>272</v>
-      </c>
-      <c r="D50" s="3"/>
+        <v>271</v>
+      </c>
+      <c r="D50" s="3" t="s">
+        <v>211</v>
+      </c>
       <c r="E50" s="3"/>
       <c r="F50" s="3"/>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A51" s="12" t="s">
         <v>18</v>
       </c>
@@ -4627,13 +5026,13 @@
         <v>46278</v>
       </c>
       <c r="C51" s="12" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
       <c r="D51" s="3"/>
       <c r="E51" s="3"/>
       <c r="F51" s="3"/>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A52" s="12" t="s">
         <v>18</v>
       </c>
@@ -4641,13 +5040,19 @@
         <v>46279</v>
       </c>
       <c r="C52" s="12" t="s">
-        <v>267</v>
-      </c>
-      <c r="D52" s="3"/>
-      <c r="E52" s="3"/>
-      <c r="F52" s="3"/>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+        <v>266</v>
+      </c>
+      <c r="D52" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E52" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="F52" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A53" s="12" t="s">
         <v>18</v>
       </c>
@@ -4655,13 +5060,19 @@
         <v>46280</v>
       </c>
       <c r="C53" s="12" t="s">
-        <v>268</v>
-      </c>
-      <c r="D53" s="3"/>
-      <c r="E53" s="3"/>
-      <c r="F53" s="3"/>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+        <v>267</v>
+      </c>
+      <c r="D53" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E53" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="F53" s="3" t="s">
+        <v>211</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.45">
       <c r="A54" s="12" t="s">
         <v>18</v>
       </c>
@@ -4669,11 +5080,17 @@
         <v>46281</v>
       </c>
       <c r="C54" s="12" t="s">
-        <v>269</v>
-      </c>
-      <c r="D54" s="3"/>
-      <c r="E54" s="3"/>
-      <c r="F54" s="3"/>
+        <v>268</v>
+      </c>
+      <c r="D54" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="E54" s="3" t="s">
+        <v>211</v>
+      </c>
+      <c r="F54" s="3" t="s">
+        <v>211</v>
+      </c>
     </row>
   </sheetData>
   <mergeCells count="1">
@@ -4687,30 +5104,30 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0100-000000000000}">
   <dimension ref="A1:H16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="2" width="20" customWidth="1"/>
     <col min="3" max="3" width="8" customWidth="1"/>
-    <col min="4" max="4" width="43.21875" customWidth="1"/>
-    <col min="5" max="5" width="15.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="8.88671875" style="21" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.5546875" style="21" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="43.19921875" customWidth="1"/>
+    <col min="5" max="5" width="15.3984375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="8.86328125" style="21" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.59765625" style="21" bestFit="1" customWidth="1"/>
     <col min="8" max="8" width="52" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="46" t="s">
+    <row r="1" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="48" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51"/>
-      <c r="E1" s="51"/>
-      <c r="F1" s="52"/>
-      <c r="G1" s="52"/>
-      <c r="H1" s="51"/>
-    </row>
-    <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="49"/>
+      <c r="G1" s="49"/>
+      <c r="H1" s="47"/>
+    </row>
+    <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>21</v>
       </c>
@@ -4736,7 +5153,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="23.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="22" t="s">
         <v>8</v>
       </c>
@@ -4762,7 +5179,7 @@
         <v>31</v>
       </c>
     </row>
-    <row r="4" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="22" t="s">
         <v>10</v>
       </c>
@@ -4786,7 +5203,7 @@
       </c>
       <c r="H4" s="13"/>
     </row>
-    <row r="5" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="22" t="s">
         <v>13</v>
       </c>
@@ -4810,7 +5227,7 @@
       </c>
       <c r="H5" s="13"/>
     </row>
-    <row r="6" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A6" s="22" t="s">
         <v>14</v>
       </c>
@@ -4834,7 +5251,7 @@
       </c>
       <c r="H6" s="13"/>
     </row>
-    <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A7" s="22" t="s">
         <v>15</v>
       </c>
@@ -4858,7 +5275,7 @@
       </c>
       <c r="H7" s="13"/>
     </row>
-    <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A8" s="9" t="s">
         <v>8</v>
       </c>
@@ -4882,7 +5299,7 @@
       </c>
       <c r="H8" s="14"/>
     </row>
-    <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A9" s="9" t="s">
         <v>10</v>
       </c>
@@ -4906,7 +5323,7 @@
       </c>
       <c r="H9" s="14"/>
     </row>
-    <row r="10" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A10" s="9" t="s">
         <v>14</v>
       </c>
@@ -4930,7 +5347,7 @@
       </c>
       <c r="H10" s="14"/>
     </row>
-    <row r="11" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A11" s="9" t="s">
         <v>15</v>
       </c>
@@ -4954,7 +5371,7 @@
       </c>
       <c r="H11" s="14"/>
     </row>
-    <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" s="11" t="s">
         <v>8</v>
       </c>
@@ -4978,7 +5395,7 @@
       </c>
       <c r="H12" s="15"/>
     </row>
-    <row r="13" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A13" s="11" t="s">
         <v>14</v>
       </c>
@@ -5002,7 +5419,7 @@
       </c>
       <c r="H13" s="15"/>
     </row>
-    <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A14" s="11" t="s">
         <v>15</v>
       </c>
@@ -5026,17 +5443,17 @@
       </c>
       <c r="H14" s="15"/>
     </row>
-    <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A16" s="50" t="s">
+    <row r="16" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A16" s="46" t="s">
         <v>44</v>
       </c>
-      <c r="B16" s="51"/>
-      <c r="C16" s="51"/>
-      <c r="D16" s="51"/>
-      <c r="E16" s="51"/>
-      <c r="F16" s="52"/>
-      <c r="G16" s="52"/>
-      <c r="H16" s="51"/>
+      <c r="B16" s="47"/>
+      <c r="C16" s="47"/>
+      <c r="D16" s="47"/>
+      <c r="E16" s="47"/>
+      <c r="F16" s="49"/>
+      <c r="G16" s="49"/>
+      <c r="H16" s="47"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -5051,15 +5468,15 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0200-000000000000}">
   <dimension ref="A1:L14"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="15.6640625" customWidth="1"/>
-    <col min="2" max="2" width="13.44140625" customWidth="1"/>
+    <col min="2" max="2" width="13.3984375" customWidth="1"/>
     <col min="3" max="8" width="15.6640625" customWidth="1"/>
     <col min="9" max="11" width="14.6640625" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="26.25" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:12" ht="26.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" s="24" t="s">
         <v>45</v>
       </c>
@@ -5094,7 +5511,7 @@
         <v>54</v>
       </c>
     </row>
-    <row r="2" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A2" s="3" t="s">
         <v>55</v>
       </c>
@@ -5132,7 +5549,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="3" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A3" s="3" t="s">
         <v>55</v>
       </c>
@@ -5170,7 +5587,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="4" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A4" s="3" t="s">
         <v>55</v>
       </c>
@@ -5208,7 +5625,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="5" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A5" s="3" t="s">
         <v>63</v>
       </c>
@@ -5243,7 +5660,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A6" s="3" t="s">
         <v>65</v>
       </c>
@@ -5278,7 +5695,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="7" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A7" s="3" t="s">
         <v>66</v>
       </c>
@@ -5313,7 +5730,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="8" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A8" s="3" t="s">
         <v>68</v>
       </c>
@@ -5348,7 +5765,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="9" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A9" s="3" t="s">
         <v>69</v>
       </c>
@@ -5383,7 +5800,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="10" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A10" s="3" t="s">
         <v>69</v>
       </c>
@@ -5418,7 +5835,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="11" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A11" s="3" t="s">
         <v>69</v>
       </c>
@@ -5453,7 +5870,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="12" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A12" s="3" t="s">
         <v>70</v>
       </c>
@@ -5488,7 +5905,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="13" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A13" s="3" t="s">
         <v>71</v>
       </c>
@@ -5523,7 +5940,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="1:12" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:12" x14ac:dyDescent="0.45">
       <c r="A14" s="3" t="s">
         <v>72</v>
       </c>
@@ -5566,26 +5983,26 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0300-000000000000}">
   <dimension ref="A1:H7"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="12" customWidth="1"/>
     <col min="3" max="3" width="14" customWidth="1"/>
     <col min="4" max="5" width="12" customWidth="1"/>
-    <col min="6" max="6" width="18.21875" customWidth="1"/>
+    <col min="6" max="6" width="18.265625" customWidth="1"/>
     <col min="7" max="7" width="18" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="46"/>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51"/>
-      <c r="E1" s="51"/>
-      <c r="F1" s="51"/>
-      <c r="G1" s="51"/>
-    </row>
-    <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:8" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="48"/>
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+      <c r="F1" s="47"/>
+      <c r="G1" s="47"/>
+    </row>
+    <row r="2" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -5608,7 +6025,7 @@
         <v>80</v>
       </c>
     </row>
-    <row r="3" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="6" t="s">
         <v>9</v>
       </c>
@@ -5630,7 +6047,7 @@
       </c>
       <c r="G3" s="3"/>
     </row>
-    <row r="4" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="10" t="s">
         <v>17</v>
       </c>
@@ -5652,7 +6069,7 @@
       </c>
       <c r="G4" s="3"/>
     </row>
-    <row r="5" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="12" t="s">
         <v>18</v>
       </c>
@@ -5674,17 +6091,17 @@
       </c>
       <c r="G5" s="3"/>
     </row>
-    <row r="7" spans="1:8" x14ac:dyDescent="0.3">
-      <c r="A7" s="50" t="s">
+    <row r="7" spans="1:8" x14ac:dyDescent="0.45">
+      <c r="A7" s="46" t="s">
         <v>81</v>
       </c>
-      <c r="B7" s="51"/>
-      <c r="C7" s="51"/>
-      <c r="D7" s="51"/>
-      <c r="E7" s="51"/>
-      <c r="F7" s="51"/>
-      <c r="G7" s="51"/>
-      <c r="H7" s="51"/>
+      <c r="B7" s="47"/>
+      <c r="C7" s="47"/>
+      <c r="D7" s="47"/>
+      <c r="E7" s="47"/>
+      <c r="F7" s="47"/>
+      <c r="G7" s="47"/>
+      <c r="H7" s="47"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -5699,15 +6116,15 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C99907B7-CFAF-4F14-AC94-4260159A2BE9}">
   <dimension ref="A1:G19"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="2" max="2" width="11" style="31" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="10.5546875" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="11.44140625" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="9.77734375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="10.53125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="11.46484375" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="9.796875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A1" s="29" t="s">
         <v>3</v>
       </c>
@@ -5730,7 +6147,7 @@
         <v>205</v>
       </c>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A2" t="s">
         <v>9</v>
       </c>
@@ -5753,7 +6170,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
         <v>9</v>
       </c>
@@ -5776,7 +6193,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A4" t="s">
         <v>9</v>
       </c>
@@ -5799,7 +6216,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
         <v>9</v>
       </c>
@@ -5822,7 +6239,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A6" t="s">
         <v>9</v>
       </c>
@@ -5845,7 +6262,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A7" t="s">
         <v>9</v>
       </c>
@@ -5865,7 +6282,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A8" t="s">
         <v>9</v>
       </c>
@@ -5885,7 +6302,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A9" t="s">
         <v>17</v>
       </c>
@@ -5908,7 +6325,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A10" t="s">
         <v>17</v>
       </c>
@@ -5931,7 +6348,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A11" t="s">
         <v>17</v>
       </c>
@@ -5954,7 +6371,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
         <v>17</v>
       </c>
@@ -5974,7 +6391,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A13" t="s">
         <v>17</v>
       </c>
@@ -5994,7 +6411,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A14" t="s">
         <v>18</v>
       </c>
@@ -6017,7 +6434,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
         <v>18</v>
       </c>
@@ -6040,7 +6457,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A16" t="s">
         <v>18</v>
       </c>
@@ -6063,7 +6480,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
         <v>18</v>
       </c>
@@ -6086,7 +6503,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A18" t="s">
         <v>18</v>
       </c>
@@ -6106,7 +6523,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:7" x14ac:dyDescent="0.45">
       <c r="A19" t="s">
         <v>18</v>
       </c>
@@ -6134,21 +6551,21 @@
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0400-000000000000}">
   <dimension ref="A1:C5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="8" customWidth="1"/>
     <col min="2" max="2" width="28" customWidth="1"/>
     <col min="3" max="3" width="35" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="46" t="s">
+    <row r="1" spans="1:3" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="48" t="s">
         <v>82</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
-    </row>
-    <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+    </row>
+    <row r="2" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>3</v>
       </c>
@@ -6159,7 +6576,7 @@
         <v>27</v>
       </c>
     </row>
-    <row r="3" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="6" t="s">
         <v>9</v>
       </c>
@@ -6168,7 +6585,7 @@
       </c>
       <c r="C3" s="13"/>
     </row>
-    <row r="4" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="6" t="s">
         <v>17</v>
       </c>
@@ -6177,7 +6594,7 @@
       </c>
       <c r="C4" s="13"/>
     </row>
-    <row r="5" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:3" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="6" t="s">
         <v>18</v>
       </c>
@@ -6198,25 +6615,25 @@
 <file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0600-000000000000}">
   <dimension ref="A1:E5"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
     <col min="1" max="1" width="6" customWidth="1"/>
-    <col min="2" max="2" width="28.77734375" customWidth="1"/>
-    <col min="3" max="3" width="34.109375" customWidth="1"/>
+    <col min="2" max="2" width="28.796875" customWidth="1"/>
+    <col min="3" max="3" width="34.1328125" customWidth="1"/>
     <col min="4" max="4" width="18" customWidth="1"/>
-    <col min="5" max="5" width="35.88671875" customWidth="1"/>
+    <col min="5" max="5" width="35.9296875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="46" t="s">
+    <row r="1" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="48" t="s">
         <v>94</v>
       </c>
-      <c r="B1" s="51"/>
-      <c r="C1" s="51"/>
-      <c r="D1" s="51"/>
-      <c r="E1" s="51"/>
-    </row>
-    <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="B1" s="47"/>
+      <c r="C1" s="47"/>
+      <c r="D1" s="47"/>
+      <c r="E1" s="47"/>
+    </row>
+    <row r="2" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A2" s="1" t="s">
         <v>95</v>
       </c>
@@ -6233,7 +6650,7 @@
         <v>99</v>
       </c>
     </row>
-    <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" s="18" t="s">
         <v>100</v>
       </c>
@@ -6250,7 +6667,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="4" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" ht="25.5" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A4" s="19" t="s">
         <v>104</v>
       </c>
@@ -6267,7 +6684,7 @@
         <v>103</v>
       </c>
     </row>
-    <row r="5" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" ht="15" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A5" s="18" t="s">
         <v>108</v>
       </c>
@@ -6295,34 +6712,34 @@
 
 <file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0500-000000000000}">
-  <dimension ref="A1:G22"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:E40"/>
+  <sheetFormatPr defaultColWidth="8.6640625" defaultRowHeight="14.25" x14ac:dyDescent="0.45"/>
   <cols>
-    <col min="1" max="1" width="10.77734375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="10.73046875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="14" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="13.21875" bestFit="1" customWidth="1"/>
-    <col min="4" max="5" width="9.109375"/>
+    <col min="3" max="3" width="13.265625" bestFit="1" customWidth="1"/>
+    <col min="4" max="5" width="9.06640625"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="21.75" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="46" t="s">
+    <row r="1" spans="1:5" ht="21.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A1" s="48" t="s">
         <v>87</v>
       </c>
-      <c r="B1" s="46"/>
-      <c r="C1" s="46"/>
-      <c r="D1" s="46"/>
-      <c r="E1" s="46"/>
-    </row>
-    <row r="2" spans="1:7" ht="29.4" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="47" t="s">
+      <c r="B1" s="48"/>
+      <c r="C1" s="48"/>
+      <c r="D1" s="48"/>
+      <c r="E1" s="48"/>
+    </row>
+    <row r="2" spans="1:5" ht="29.35" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A2" s="50" t="s">
         <v>212</v>
       </c>
-      <c r="B2" s="47"/>
-      <c r="C2" s="47"/>
-      <c r="D2" s="47"/>
-      <c r="E2" s="47"/>
-    </row>
-    <row r="3" spans="1:7" s="25" customFormat="1" x14ac:dyDescent="0.3">
+      <c r="B2" s="50"/>
+      <c r="C2" s="50"/>
+      <c r="D2" s="50"/>
+      <c r="E2" s="50"/>
+    </row>
+    <row r="3" spans="1:5" s="25" customFormat="1" x14ac:dyDescent="0.45">
       <c r="A3" s="36" t="s">
         <v>213</v>
       </c>
@@ -6339,7 +6756,7 @@
         <v>230</v>
       </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A4" s="37" t="s">
         <v>222</v>
       </c>
@@ -6356,106 +6773,100 @@
         <v>234</v>
       </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A5" s="37" t="s">
         <v>216</v>
       </c>
-      <c r="B5" s="45">
-        <v>0.31877314814814817</v>
+      <c r="B5" s="37" t="s">
+        <v>276</v>
       </c>
       <c r="C5" s="38" t="s">
-        <v>157</v>
+        <v>179</v>
       </c>
       <c r="D5" s="39">
-        <v>1000</v>
+        <v>500</v>
       </c>
       <c r="E5" s="37" t="s">
         <v>234</v>
       </c>
-      <c r="G5" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A6" s="37" t="s">
         <v>216</v>
       </c>
-      <c r="B6" s="45">
-        <v>0.32085648148148149</v>
+      <c r="B6" s="37" t="s">
+        <v>249</v>
       </c>
       <c r="C6" s="38" t="s">
-        <v>189</v>
+        <v>90</v>
       </c>
       <c r="D6" s="39">
         <v>1600</v>
       </c>
       <c r="E6" s="37" t="s">
-        <v>233</v>
-      </c>
-      <c r="G6" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="7" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A7" s="37" t="s">
         <v>216</v>
       </c>
-      <c r="B7" s="45">
-        <v>0.59734953703703708</v>
+      <c r="B7" s="37" t="s">
+        <v>250</v>
       </c>
       <c r="C7" s="38" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="D7" s="39">
-        <v>500</v>
+        <v>200</v>
       </c>
       <c r="E7" s="37" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="8" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A8" s="37" t="s">
         <v>216</v>
       </c>
       <c r="B8" s="37" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="C8" s="38" t="s">
-        <v>157</v>
+        <v>86</v>
       </c>
       <c r="D8" s="39">
-        <v>2000</v>
+        <v>2800</v>
       </c>
       <c r="E8" s="37" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A9" s="37" t="s">
         <v>216</v>
       </c>
       <c r="B9" s="37" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="C9" s="38" t="s">
-        <v>90</v>
+        <v>166</v>
       </c>
       <c r="D9" s="39">
-        <v>1600</v>
+        <v>1000</v>
       </c>
       <c r="E9" s="37" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="10" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A10" s="37" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B10" s="37" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="C10" s="38" t="s">
-        <v>177</v>
+        <v>86</v>
       </c>
       <c r="D10" s="39">
         <v>200</v>
@@ -6464,212 +6875,518 @@
         <v>233</v>
       </c>
     </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A11" s="37" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B11" s="37" t="s">
-        <v>252</v>
+        <v>279</v>
       </c>
       <c r="C11" s="38" t="s">
-        <v>86</v>
+        <v>189</v>
       </c>
       <c r="D11" s="39">
-        <v>2800</v>
+        <v>1600</v>
       </c>
       <c r="E11" s="37" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A12" s="37" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="B12" s="37" t="s">
-        <v>253</v>
+        <v>280</v>
       </c>
       <c r="C12" s="38" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="D12" s="39">
-        <v>1000</v>
+        <v>600</v>
       </c>
       <c r="E12" s="37" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A13" s="44">
-        <v>46267</v>
-      </c>
-      <c r="B13" s="45">
-        <v>0.93065972222222226</v>
+    <row r="13" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A13" s="37" t="s">
+        <v>217</v>
+      </c>
+      <c r="B13" s="37" t="s">
+        <v>254</v>
       </c>
       <c r="C13" s="38" t="s">
-        <v>189</v>
+        <v>167</v>
       </c>
       <c r="D13" s="39">
-        <v>1600</v>
+        <v>3000</v>
       </c>
       <c r="E13" s="37" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="14" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A14" s="37" t="s">
+        <v>218</v>
+      </c>
+      <c r="B14" s="37" t="s">
+        <v>255</v>
+      </c>
+      <c r="C14" s="38" t="s">
+        <v>148</v>
+      </c>
+      <c r="D14" s="39">
+        <v>600</v>
+      </c>
+      <c r="E14" s="37" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="15" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A15" s="37" t="s">
+        <v>218</v>
+      </c>
+      <c r="B15" s="37" t="s">
+        <v>256</v>
+      </c>
+      <c r="C15" s="38" t="s">
+        <v>86</v>
+      </c>
+      <c r="D15" s="39">
+        <v>400</v>
+      </c>
+      <c r="E15" s="37" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A14" s="37" t="s">
-        <v>217</v>
-      </c>
-      <c r="B14" s="37" t="s">
-        <v>254</v>
-      </c>
-      <c r="C14" s="38" t="s">
-        <v>86</v>
-      </c>
-      <c r="D14" s="39">
-        <v>200</v>
-      </c>
-      <c r="E14" s="37" t="s">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A16" s="37" t="s">
+        <v>219</v>
+      </c>
+      <c r="B16" s="37" t="s">
+        <v>257</v>
+      </c>
+      <c r="C16" s="38" t="s">
+        <v>178</v>
+      </c>
+      <c r="D16" s="39">
+        <v>1200</v>
+      </c>
+      <c r="E16" s="37" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A15" s="37" t="s">
-        <v>217</v>
-      </c>
-      <c r="B15" s="45">
-        <v>0.19550925925925927</v>
-      </c>
-      <c r="C15" s="38" t="s">
-        <v>165</v>
-      </c>
-      <c r="D15" s="39">
-        <v>600</v>
-      </c>
-      <c r="E15" s="37" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="A16" s="37" t="s">
-        <v>217</v>
-      </c>
-      <c r="B16" s="37" t="s">
-        <v>255</v>
-      </c>
-      <c r="C16" s="38" t="s">
-        <v>167</v>
-      </c>
-      <c r="D16" s="39">
-        <v>3000</v>
-      </c>
-      <c r="E16" s="37" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A17" s="37" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B17" s="37" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="C17" s="38" t="s">
-        <v>148</v>
+        <v>163</v>
       </c>
       <c r="D17" s="39">
-        <v>600</v>
+        <v>1200</v>
       </c>
       <c r="E17" s="37" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A18" s="37" t="s">
-        <v>218</v>
+        <v>220</v>
       </c>
       <c r="B18" s="37" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="C18" s="38" t="s">
-        <v>86</v>
+        <v>177</v>
       </c>
       <c r="D18" s="39">
-        <v>400</v>
+        <v>2200</v>
       </c>
       <c r="E18" s="37" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A19" s="37" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="B19" s="37" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="C19" s="38" t="s">
-        <v>178</v>
+        <v>89</v>
       </c>
       <c r="D19" s="39">
-        <v>1200</v>
+        <v>2400</v>
       </c>
       <c r="E19" s="37" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.45">
       <c r="A20" s="37" t="s">
-        <v>220</v>
+        <v>221</v>
       </c>
       <c r="B20" s="37" t="s">
-        <v>259</v>
+        <v>281</v>
       </c>
       <c r="C20" s="38" t="s">
-        <v>163</v>
+        <v>178</v>
       </c>
       <c r="D20" s="39">
         <v>1200</v>
       </c>
       <c r="E20" s="37" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A21" s="37" t="s">
+        <v>282</v>
+      </c>
+      <c r="B21" s="37" t="s">
+        <v>283</v>
+      </c>
+      <c r="C21" s="38" t="s">
+        <v>90</v>
+      </c>
+      <c r="D21" s="39">
+        <v>1000</v>
+      </c>
+      <c r="E21" s="37" t="s">
         <v>234</v>
       </c>
     </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="37" t="s">
-        <v>220</v>
-      </c>
-      <c r="B21" s="37" t="s">
-        <v>260</v>
-      </c>
-      <c r="C21" s="38" t="s">
-        <v>177</v>
-      </c>
-      <c r="D21" s="39">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A22" s="37" t="s">
+        <v>282</v>
+      </c>
+      <c r="B22" s="37" t="s">
+        <v>284</v>
+      </c>
+      <c r="C22" s="38" t="s">
+        <v>85</v>
+      </c>
+      <c r="D22" s="39">
+        <v>800</v>
+      </c>
+      <c r="E22" s="37" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A23" s="37" t="s">
+        <v>282</v>
+      </c>
+      <c r="B23" s="37" t="s">
+        <v>285</v>
+      </c>
+      <c r="C23" s="38" t="s">
+        <v>88</v>
+      </c>
+      <c r="D23" s="39">
+        <v>1000</v>
+      </c>
+      <c r="E23" s="37" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A24" s="37" t="s">
+        <v>282</v>
+      </c>
+      <c r="B24" s="37" t="s">
+        <v>286</v>
+      </c>
+      <c r="C24" s="38" t="s">
+        <v>167</v>
+      </c>
+      <c r="D24" s="39">
+        <v>3000</v>
+      </c>
+      <c r="E24" s="37" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A25" s="37" t="s">
+        <v>287</v>
+      </c>
+      <c r="B25" s="37" t="s">
+        <v>288</v>
+      </c>
+      <c r="C25" s="38" t="s">
+        <v>86</v>
+      </c>
+      <c r="D25" s="39">
+        <v>1600</v>
+      </c>
+      <c r="E25" s="37" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A26" s="37" t="s">
+        <v>287</v>
+      </c>
+      <c r="B26" s="37" t="s">
+        <v>289</v>
+      </c>
+      <c r="C26" s="38" t="s">
+        <v>179</v>
+      </c>
+      <c r="D26" s="39">
+        <v>1600</v>
+      </c>
+      <c r="E26" s="37" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A27" s="37" t="s">
+        <v>287</v>
+      </c>
+      <c r="B27" s="37" t="s">
+        <v>290</v>
+      </c>
+      <c r="C27" s="38" t="s">
+        <v>157</v>
+      </c>
+      <c r="D27" s="39">
+        <v>900</v>
+      </c>
+      <c r="E27" s="37" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A28" s="37" t="s">
+        <v>291</v>
+      </c>
+      <c r="B28" s="37" t="s">
+        <v>292</v>
+      </c>
+      <c r="C28" s="38" t="s">
+        <v>153</v>
+      </c>
+      <c r="D28" s="39">
+        <v>2600</v>
+      </c>
+      <c r="E28" s="37" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A29" s="37" t="s">
+        <v>293</v>
+      </c>
+      <c r="B29" s="37" t="s">
+        <v>294</v>
+      </c>
+      <c r="C29" s="38" t="s">
+        <v>187</v>
+      </c>
+      <c r="D29" s="39">
+        <v>1000</v>
+      </c>
+      <c r="E29" s="37" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A30" s="37" t="s">
+        <v>293</v>
+      </c>
+      <c r="B30" s="37" t="s">
+        <v>295</v>
+      </c>
+      <c r="C30" s="38" t="s">
+        <v>157</v>
+      </c>
+      <c r="D30" s="39">
+        <v>2400</v>
+      </c>
+      <c r="E30" s="37" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A31" s="37" t="s">
+        <v>293</v>
+      </c>
+      <c r="B31" s="37" t="s">
+        <v>296</v>
+      </c>
+      <c r="C31" s="38" t="s">
+        <v>188</v>
+      </c>
+      <c r="D31" s="39">
         <v>2200</v>
       </c>
-      <c r="E21" s="37" t="s">
+      <c r="E31" s="37" t="s">
         <v>233</v>
       </c>
     </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A22" s="37" t="s">
-        <v>221</v>
-      </c>
-      <c r="B22" s="37" t="s">
-        <v>261</v>
-      </c>
-      <c r="C22" s="38" t="s">
+    <row r="32" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A32" s="37" t="s">
+        <v>297</v>
+      </c>
+      <c r="B32" s="37" t="s">
+        <v>298</v>
+      </c>
+      <c r="C32" s="38" t="s">
+        <v>153</v>
+      </c>
+      <c r="D32" s="39">
+        <v>800</v>
+      </c>
+      <c r="E32" s="37" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A33" s="37" t="s">
+        <v>297</v>
+      </c>
+      <c r="B33" s="37" t="s">
+        <v>299</v>
+      </c>
+      <c r="C33" s="38" t="s">
+        <v>84</v>
+      </c>
+      <c r="D33" s="39">
+        <v>600</v>
+      </c>
+      <c r="E33" s="37" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A34" s="37" t="s">
+        <v>297</v>
+      </c>
+      <c r="B34" s="37" t="s">
+        <v>300</v>
+      </c>
+      <c r="C34" s="38" t="s">
+        <v>149</v>
+      </c>
+      <c r="D34" s="39">
+        <v>200</v>
+      </c>
+      <c r="E34" s="37" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A35" s="37" t="s">
+        <v>297</v>
+      </c>
+      <c r="B35" s="37" t="s">
+        <v>301</v>
+      </c>
+      <c r="C35" s="38" t="s">
+        <v>167</v>
+      </c>
+      <c r="D35" s="39">
+        <v>2600</v>
+      </c>
+      <c r="E35" s="37" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A36" s="37" t="s">
+        <v>302</v>
+      </c>
+      <c r="B36" s="37" t="s">
+        <v>303</v>
+      </c>
+      <c r="C36" s="38" t="s">
+        <v>163</v>
+      </c>
+      <c r="D36" s="39">
+        <v>1200</v>
+      </c>
+      <c r="E36" s="37" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="37" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A37" s="37" t="s">
+        <v>302</v>
+      </c>
+      <c r="B37" s="37" t="s">
+        <v>304</v>
+      </c>
+      <c r="C37" s="38" t="s">
+        <v>90</v>
+      </c>
+      <c r="D37" s="39">
+        <v>2000</v>
+      </c>
+      <c r="E37" s="37" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="38" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A38" s="37" t="s">
+        <v>302</v>
+      </c>
+      <c r="B38" s="37" t="s">
+        <v>305</v>
+      </c>
+      <c r="C38" s="38" t="s">
+        <v>179</v>
+      </c>
+      <c r="D38" s="39">
+        <v>400</v>
+      </c>
+      <c r="E38" s="37" t="s">
+        <v>234</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A39" s="37" t="s">
+        <v>302</v>
+      </c>
+      <c r="B39" s="37" t="s">
+        <v>306</v>
+      </c>
+      <c r="C39" s="38" t="s">
         <v>89</v>
       </c>
-      <c r="D22" s="39">
-        <v>2400</v>
-      </c>
-      <c r="E22" s="37" t="s">
+      <c r="D39" s="39">
+        <v>1000</v>
+      </c>
+      <c r="E39" s="37" t="s">
         <v>233</v>
       </c>
     </row>
+    <row r="40" spans="1:5" x14ac:dyDescent="0.45">
+      <c r="A40" s="37" t="s">
+        <v>302</v>
+      </c>
+      <c r="B40" s="37" t="s">
+        <v>307</v>
+      </c>
+      <c r="C40" s="38" t="s">
+        <v>91</v>
+      </c>
+      <c r="D40" s="39">
+        <v>800</v>
+      </c>
+      <c r="E40" s="37" t="s">
+        <v>233</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A3:E22" xr:uid="{00000000-0001-0000-0500-000000000000}"/>
+  <autoFilter ref="A3:E8" xr:uid="{00000000-0001-0000-0500-000000000000}"/>
   <mergeCells count="2">
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="A2:E2"/>

</xml_diff>